<commit_message>
fix: use US locale currency formats and honor file numFmt overrides instead of ALL_LANGUAGES ￥ entries
getBuiltinFormat resolved BUILTIN_FORMATS_ALL_LANGUAGES before the
locale table and before the caller-provided format, so US-locale readers
got the all-language ￥ currency entries at indices 5-8/42/44 and the
file's own styles.xml numFmt override was outranked (POI bug 49928
behavior). Skip the all-language shortcut when the locale resolves to
the US table, so the per-file format and the US $ entries win. CN and
default (null) locale behavior is unchanged.

Update the two dataformat fixture dateStringUs cells that recorded the
old CN-flavored rendering of built-in date formats 14/22 under
Locale.US; the CN and number expectations are untouched.
</commit_message>
<xml_diff>
--- a/fesod-sheet/src/test/resources/dataformat/dataformat.xlsx
+++ b/fesod-sheet/src/test/resources/dataformat/dataformat.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11028"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuangjiaju/IdeaProjects/easyexcel/easyexcel-test/src/test/resources/dataformat/"/>
     </mc:Choice>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="58">
   <si>
     <t>date</t>
   </si>
@@ -198,6 +198,12 @@
   </si>
   <si>
     <t>1月</t>
+  </si>
+  <si>
+    <t>1/1/20 1:01</t>
+  </si>
+  <si>
+    <t>1/1/20</t>
   </si>
 </sst>
 </file>
@@ -750,15 +756,15 @@
   <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="26.1640625" customWidth="1"/>
-    <col min="2" max="4" width="22.5" style="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="26.1640625"/>
+    <col min="2" max="4" customWidth="true" style="1" width="22.5"/>
     <col min="5" max="5" width="10.33203125"/>
-    <col min="6" max="6" width="22.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="18" style="1" customWidth="1"/>
+    <col min="6" max="6" customWidth="true" style="1" width="22.6640625"/>
+    <col min="7" max="7" customWidth="true" style="1" width="18.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -770,7 +776,7 @@
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -788,9 +794,9 @@
         <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2">
+        <v>56</v>
+      </c>
+      <c r="E2" s="0">
         <v>1.1111</v>
       </c>
       <c r="F2" s="1" t="s">
@@ -828,7 +834,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="E4" s="6">
         <v>1.1111</v>
@@ -1010,7 +1016,7 @@
       <c r="D13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="0">
         <v>1</v>
       </c>
       <c r="F13" s="1" t="s">

</xml_diff>

<commit_message>
fix: only skip the all-language builtin format where the locale table differs
</commit_message>
<xml_diff>
--- a/fesod-sheet/src/test/resources/dataformat/dataformat.xlsx
+++ b/fesod-sheet/src/test/resources/dataformat/dataformat.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11028"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuangjiaju/IdeaProjects/easyexcel/easyexcel-test/src/test/resources/dataformat/"/>
     </mc:Choice>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="56">
   <si>
     <t>date</t>
   </si>
@@ -198,12 +198,6 @@
   </si>
   <si>
     <t>1月</t>
-  </si>
-  <si>
-    <t>1/1/20 1:01</t>
-  </si>
-  <si>
-    <t>1/1/20</t>
   </si>
 </sst>
 </file>
@@ -756,15 +750,15 @@
   <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="26.1640625"/>
-    <col min="2" max="4" customWidth="true" style="1" width="22.5"/>
+    <col min="1" max="1" width="26.1640625" customWidth="1"/>
+    <col min="2" max="4" width="22.5" style="1" customWidth="1"/>
     <col min="5" max="5" width="10.33203125"/>
-    <col min="6" max="6" customWidth="true" style="1" width="22.6640625"/>
-    <col min="7" max="7" customWidth="true" style="1" width="18.0"/>
+    <col min="6" max="6" width="22.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="18" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -776,7 +770,7 @@
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -794,9 +788,9 @@
         <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E2" s="0">
+        <v>6</v>
+      </c>
+      <c r="E2">
         <v>1.1111</v>
       </c>
       <c r="F2" s="1" t="s">
@@ -834,7 +828,7 @@
         <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="E4" s="6">
         <v>1.1111</v>
@@ -1016,7 +1010,7 @@
       <c r="D13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="0">
+      <c r="E13">
         <v>1</v>
       </c>
       <c r="F13" s="1" t="s">

</xml_diff>